<commit_message>
Update messages file (adapted demographics)
</commit_message>
<xml_diff>
--- a/PsychoPy-online/fpjt_files/Messages.xlsx
+++ b/PsychoPy-online/fpjt_files/Messages.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cdabb12e9f34f4c5/10_Paper/105_MIA/10_BAS_Collab/FPJT/PsychoPy-online/fpjt_files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cdabb12e9f34f4c5/10_Paper/111_MIA_validation/02_Experiment/PsychoPy-online/fpjt_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="252" documentId="8_{9A5DEF40-44A6-4D82-8A38-CC73A1DAE49D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{017C1BFF-8D4B-4688-B369-D5E1ACE56321}"/>
+  <xr:revisionPtr revIDLastSave="255" documentId="8_{9A5DEF40-44A6-4D82-8A38-CC73A1DAE49D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{200C2857-4080-4FCE-9330-149F2BAEAE8D}"/>
   <bookViews>
-    <workbookView xWindow="44880" yWindow="11850" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14476" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -622,579 +622,579 @@
 Lever le bras gauche vers l’avant dans la direction du regard &amp; faire pivoter le haut du corps vers la gauche ==&gt;</t>
   </si>
   <si>
-    <t>You will now hear an audio instruction in 36 trials, each containing 3 to 7 consecutive movements. IMAGINE what it LOOKS LIKE and how it FEELS to perform these movements YOURSELF. Remain seated calmly, CLOSE YOUR EYES and DO NOT MOVE.
+    <t>When making your decision, pay attention to the rotation of the upper body and to the position of the head, arms, and legs.
+Because the movements build on each other, make sure that when you ROTATE YOUR UPPER BODY, your ARMS and your HEAD ROTATE WITH IT. Your LEGS do NOT rotate.</t>
+  </si>
+  <si>
+    <t>Dies ist das Ende des Experiments.
+Vielen Dank für Ihre Teilnahme!
+Das Experiment schließt sich in 3 Sekunden.</t>
+  </si>
+  <si>
+    <t>Al tomar su decisión, preste atención a la rotación del tronco, así como a la posición de la cabeza, los brazos y las piernas.
+Dado que los movimientos se encadenan, asegúrese de que, cuando GIRE EL TRONCO, los BRAZOS y la CABEZA GIREN TAMBIÉN. Las PIERNAS, en cambio, NO giran.</t>
+  </si>
+  <si>
+    <t>Ceci est la fin de l’expérience.
+Merci pour votre participation.
+L’expérience se terminera dans 3 secondes.</t>
+  </si>
+  <si>
+    <t>Lors de votre décision, prêtez attention à la rotation du haut du corps ainsi qu’à la position de la tête, des bras et des jambes.
+Étant donné que les mouvements s’enchaînent, veillez à ce que, lorsque vous EFFECTUEZ UNE ROTATION DU HAUT DU CORPS, les BRAS et la TÊTE TOURNENT ÉGALEMENT. Les JAMBES, en revanche, ne tournent PAS.</t>
+  </si>
+  <si>
+    <t>Es folgen nun 4 Übungsdurchgänge.</t>
+  </si>
+  <si>
+    <t>Positionieren Sie Ihre Zeigefinger nun auf den Tasten ‚S‘ und ‚L‘ .
+Lassen Sie Ihre Finger auf diesen Tasten ruhen, bis Sie alle Durchgänge der Aufgabe absolviert haben.
+Wenn Sie bereit sind, drücken Sie mit Ihrem Daumen die Leertaste.</t>
+  </si>
+  <si>
+    <t>task_instr_msg_3_bimanual</t>
+  </si>
+  <si>
+    <t>task_instr_msg_3_left</t>
+  </si>
+  <si>
+    <t>task_instr_msg_3_right</t>
+  </si>
+  <si>
+    <t>pract_instr_msg</t>
+  </si>
+  <si>
+    <t>testbl_instr_msg</t>
+  </si>
+  <si>
+    <t>no_feedback_msg</t>
+  </si>
+  <si>
+    <t>Sie werden nun keine Rückmeldungen mehr erhalten.</t>
+  </si>
+  <si>
+    <t>reminder_msg</t>
+  </si>
+  <si>
+    <t>Erinnerung:
+Stellen Sie sich vor, WIE ES AUSSIEHT und WIE ES SICH ANFÜHLT, die in der Audioinstruktion beschriebenen Bewegungen selbst auszuführen.
+Öffnen Sie Ihre Augen beim Signalton. Entscheiden Sie so SCHNELL UND KORREKT wie möglich, ob das gezeigte Bild zu der Endposition in Ihrer Vorstellung passt.</t>
+  </si>
+  <si>
+    <t>There will now be 4 practice trials.</t>
+  </si>
+  <si>
+    <t>Now place your index fingers on the ‘S’ and ‘L’ keys.
+Keep your fingers resting on these keys until you have completed all trials of the task.
+When you are ready, press the space bar with your thumb.</t>
+  </si>
+  <si>
+    <t>Positionieren Sie Mittel- und Zeigefinger Ihrer linken Hand nun auf den Tasten ‚G‘ und ‚H‘ .
+Lassen Sie Ihre Finger auf diesen Tasten ruhen, bis Sie alle Durchgänge der Aufgabe absolviert haben.
+Wenn Sie bereit sind, drücken Sie mit Ihrem Daumen die Leertaste.</t>
+  </si>
+  <si>
+    <t>Positionieren Sie Zeige- und Mittelfinger Ihrer rechten Hand nun auf den Tasten ‚G‘ und ‚H‘ .
+Lassen Sie Ihre Finger auf diesen Tasten ruhen, bis Sie alle Durchgänge der Aufgabe absolviert haben.
+Wenn Sie bereit sind, drücken Sie mit Ihrem Daumen die Leertaste.</t>
+  </si>
+  <si>
+    <t>Now place the index and middle fingers of your left hand on the ‘G’ and ‘H’ keys.
+Keep your fingers resting on these keys until you have completed all trials of the task.
+When you are ready, press the space bar with your thumb.</t>
+  </si>
+  <si>
+    <t>Now place the index and middle fingers of your right hand on the ‘G’ and ‘H’ keys.
+Keep your fingers resting on these keys until you have completed all trials of the task.
+When you are ready, press the space bar with your thumb.</t>
+  </si>
+  <si>
+    <t>You will now receive no further feedback.</t>
+  </si>
+  <si>
+    <t>Reminder:
+Imagine WHAT IT LOOKS LIKE and HOW IT FEELS to perform the movements described in the audio instruction yourself.
+Open your eyes when you hear the signal tone. Decide as QUICKLY AND ACCURATELY as possible whether the displayed image matches the final position in your imagery.</t>
+  </si>
+  <si>
+    <t>Il va maintenant y avoir 4 essais d’entraînement.</t>
+  </si>
+  <si>
+    <t>Vous ne recevrez désormais plus aucun retour.</t>
+  </si>
+  <si>
+    <t>A continuación habrá 4 ensayos de práctica.</t>
+  </si>
+  <si>
+    <t>Coloque ahora sus dedos índices sobre las teclas “S” y “L”.
+Mantenga los dedos apoyados sobre estas teclas hasta que haya completado todos los ensayos de la tarea.
+Cuando esté listo/a, presione la barra espaciadora con el pulgar.</t>
+  </si>
+  <si>
+    <t>Coloque ahora el dedo índice y el dedo medio de su mano izquierda sobre las teclas “G” y “H”.
+Mantenga los dedos apoyados sobre estas teclas hasta que haya completado todos los ensayos de la tarea.
+Cuando esté listo/a, presione la barra espaciadora con el pulgar.</t>
+  </si>
+  <si>
+    <t>Coloque ahora el dedo índice y el dedo medio de su mano derecha sobre las teclas “G” y “H”.
+Mantenga los dedos apoyados sobre estas teclas hasta que haya completado todos los ensayos de la tarea.
+Cuando esté listo/a, presione la barra espaciadora con el pulgar.</t>
+  </si>
+  <si>
+    <t>A partir de ahora no recibirá más retroalimentación.</t>
+  </si>
+  <si>
+    <t>Recordatorio:
+Imagine CÓMO SE VE y CÓMO SE SIENTE ejecutar usted mismo/a los movimientos descritos en la instrucción auditiva.
+Abra los ojos cuando escuche la señal sonora. Decida lo más RÁPIDA Y CORRECTAMENTE posible si la imagen mostrada coincide con la posición final en su imagery.</t>
+  </si>
+  <si>
+    <t>Placez maintenant vos index sur les touches « S » et « L ».
+Laissez vos doigts reposer sur ces touches jusqu’à ce que vous ayez terminé tous les essais de la tâche.
+Lorsque vous êtes prêt(e), appuyez sur la barre d’espace avec votre pouce.</t>
+  </si>
+  <si>
+    <t>Placez maintenant l’index et le majeur de votre main gauche sur les touches « G » et « H ».
+Laissez vos doigts reposer sur ces touches jusqu’à ce que vous ayez terminé tous les essais de la tâche.
+Lorsque vous êtes prêt(e), appuyez sur la barre d’espace avec votre pouce.</t>
+  </si>
+  <si>
+    <t>Placez maintenant l’index et le majeur de votre main droite sur les touches « G » et « H ».
+Laissez vos doigts reposer sur ces touches jusqu’à ce que vous ayez terminé tous les essais de la tâche.
+Lorsque vous êtes prêt(e), appuyez sur la barre d’espace avec votre pouce.</t>
+  </si>
+  <si>
+    <t>you are supposed to imagine how the person in the picture performs the movements.</t>
+  </si>
+  <si>
+    <t>Achten Sie bei Ihrer Entscheidung auf die Drehung des Oberkörpers, die Position des Kopfes, der Arme und Beine.
+Da die Bewegungen aufeinander aufbauen, achten Sie darauf, dass Sie bei DREHUNG IHRES OBERKÖRPERS Ihre ARME und Ihren KOPF MITDREHEN. Ihre BEINE drehen sich dabei NICHT mit.</t>
+  </si>
+  <si>
+    <t>Beispiele:
+&lt;== Neigung des Kopfes nach unten &amp; Drehung des Oberkörpers nach links.
+Anheben des linken Arms in Blickrichtung nach vorne &amp; Drehung des Oberkörpers nach links ==&gt;</t>
+  </si>
+  <si>
+    <t>KORREKTE Antwort</t>
+  </si>
+  <si>
+    <t>CORRECT response</t>
+  </si>
+  <si>
+    <t>INCORRECT response</t>
+  </si>
+  <si>
+    <t>Respuesta CORRECTA</t>
+  </si>
+  <si>
+    <t>Respuesta INCORRECTA</t>
+  </si>
+  <si>
+    <t>Réponse CORRECTE</t>
+  </si>
+  <si>
+    <t>Réponse INCORRECTE</t>
+  </si>
+  <si>
+    <t>fam_msg_1a</t>
+  </si>
+  <si>
+    <t>fam_msg_1b</t>
+  </si>
+  <si>
+    <t>no_movement</t>
+  </si>
+  <si>
+    <t>In the following, you will see 16 images of a person from behind who started in this upright, standing position …</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Im Folgenden sehen Sie 16 Bilder einer Person von hinten, die in dieser aufrechten, stehenden Position startete… </t>
+  </si>
+  <si>
+    <t>A continuación, verá 16 imágenes de una persona vista desde atrás, que comenzó en esta posición erguida y de pie …</t>
+  </si>
+  <si>
+    <t>Dans ce qui suit, vous verrez 16 images d’une personne vue de dos, qui a commencé dans cette position droite et debout …</t>
+  </si>
+  <si>
+    <t>fam_msg_2</t>
+  </si>
+  <si>
+    <t>volume_calib_msg</t>
+  </si>
+  <si>
+    <t>testsound_label</t>
+  </si>
+  <si>
+    <t>In diesem Experiment werden Sie mehrere Audios anhören. Klicken Sie auf ‚Testton abspielen‘ abspielen und stellen Sie die Lautstärke an Ihrem Gerät passend ein.</t>
+  </si>
+  <si>
+    <t>Testton abspielen</t>
+  </si>
+  <si>
+    <t>In this experiment, you will listen to multiple audio recordings. Click on “Play test sound” and adjust the volume on your device accordingly.</t>
+  </si>
+  <si>
+    <t>Play test sound</t>
+  </si>
+  <si>
+    <t>En este experimento, escuchará varios audios. Haga clic en “Reproducir sonido de prueba” y ajuste el volumen de su dispositivo según sea necesario.</t>
+  </si>
+  <si>
+    <t>Reproducir sonido de prueba</t>
+  </si>
+  <si>
+    <t>Dans cette expérience, vous écouterez plusieurs enregistrements audio. Cliquez sur « Lire le son de test » et ajustez le volume de votre appareil en conséquence.</t>
+  </si>
+  <si>
+    <t>Lire le son de test</t>
+  </si>
+  <si>
+    <t>This is the end of the experiment.
+Thank you for participating!
+The experiment finishes in 3 seconds.</t>
+  </si>
+  <si>
+    <t>Este es el final del experimento.
+Gracias por su participación.
+El experimento finalizará en 3 segundos.</t>
+  </si>
+  <si>
+    <t>Unfortunately, your answers were not completely correct.
+Please read the instructions carefully again.</t>
+  </si>
+  <si>
+    <t>testsound</t>
+  </si>
+  <si>
+    <t>Stellen Sie die Lautstärke an Ihrem Gerät so ein, dass Sie dieses Audio klar und deutlich hören können. Bitte lassen Sie die Lautstärke anschließend unverändert. Drücken Sie danach die Leertaste, um fortzufahren.</t>
+  </si>
+  <si>
+    <t>Adjust the volume on your device so that you can hear this audio clearly. Please keep the volume unchanged afterwards. Then press the space bar to continue.</t>
+  </si>
+  <si>
+    <t>Réglez le volume de votre appareil de manière à entendre clairement cet audio. Veuillez ensuite laisser le volume inchangé. Appuyez ensuite sur la barre d’espace pour continuer.</t>
+  </si>
+  <si>
+    <t>Ajuste el volumen de su dispositivo para que pueda escuchar este audio con claridad. Por favor, mantenga el volumen sin cambios a continuación. Luego presione la barra espaciadora para continuar.</t>
+  </si>
+  <si>
+    <t>Raise your right arm forward in the direction of your gaze.</t>
+  </si>
+  <si>
+    <t>Raise your left arm forward in the direction of your gaze.</t>
+  </si>
+  <si>
+    <t>Examples:
+&lt;== Tilting the head downward &amp; rotating the upper body to the left.
+Raising the left arm forward in the direction of gaze &amp; rotating the upper body to the left ==&gt;</t>
+  </si>
+  <si>
+    <t>demographics_msg</t>
+  </si>
+  <si>
+    <t>Please fill out this information about yourself.</t>
+  </si>
+  <si>
+    <t>Por favor completa esta información sobre ti.</t>
+  </si>
+  <si>
+    <t>Veuillez remplir ces informations vous concernant.</t>
+  </si>
+  <si>
+    <t>Bitte füllen Sie diese Informationen über sich selbst aus.</t>
+  </si>
+  <si>
+    <t>age_msg</t>
+  </si>
+  <si>
+    <t>Age:</t>
+  </si>
+  <si>
+    <t>Edad:</t>
+  </si>
+  <si>
+    <t>Âge :</t>
+  </si>
+  <si>
+    <t>Alter:</t>
+  </si>
+  <si>
+    <t>gender_msg</t>
+  </si>
+  <si>
+    <t>Gender:</t>
+  </si>
+  <si>
+    <t>Género</t>
+  </si>
+  <si>
+    <t>Genre :</t>
+  </si>
+  <si>
+    <t>Geschlecht:</t>
+  </si>
+  <si>
+    <t>f_msg</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>Mujer</t>
+  </si>
+  <si>
+    <t>Femme</t>
+  </si>
+  <si>
+    <t>Weiblich</t>
+  </si>
+  <si>
+    <t>m_msg</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>Hombre</t>
+  </si>
+  <si>
+    <t>Homme</t>
+  </si>
+  <si>
+    <t>Männlich</t>
+  </si>
+  <si>
+    <t>tg_msg</t>
+  </si>
+  <si>
+    <t>Trans-gender</t>
+  </si>
+  <si>
+    <t>Transgénero</t>
+  </si>
+  <si>
+    <t>Transgenre</t>
+  </si>
+  <si>
+    <t>Transgender</t>
+  </si>
+  <si>
+    <t>nb_msg</t>
+  </si>
+  <si>
+    <t>Non-binary</t>
+  </si>
+  <si>
+    <t>No binario</t>
+  </si>
+  <si>
+    <t>Non binaire</t>
+  </si>
+  <si>
+    <t>Nicht-binär</t>
+  </si>
+  <si>
+    <t>o_msg</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>Otro</t>
+  </si>
+  <si>
+    <t>Autre</t>
+  </si>
+  <si>
+    <t>Sonstiges</t>
+  </si>
+  <si>
+    <t>pns_msg</t>
+  </si>
+  <si>
+    <t>Prefer not saying</t>
+  </si>
+  <si>
+    <t>Prefiero no decirlo</t>
+  </si>
+  <si>
+    <t>Préfère ne pas le dire</t>
+  </si>
+  <si>
+    <t>Möchte ich nicht sagen</t>
+  </si>
+  <si>
+    <t>next_msg</t>
+  </si>
+  <si>
+    <t>Next</t>
+  </si>
+  <si>
+    <t>Weiter</t>
+  </si>
+  <si>
+    <t>Siguiente</t>
+  </si>
+  <si>
+    <t>Suivant</t>
+  </si>
+  <si>
+    <t>laterality_msg</t>
+  </si>
+  <si>
+    <t>Hand dominance:</t>
+  </si>
+  <si>
+    <t>Mano dominante:</t>
+  </si>
+  <si>
+    <t>Dominance manuelle :</t>
+  </si>
+  <si>
+    <t>Handdominanz:</t>
+  </si>
+  <si>
+    <t>left_msg</t>
+  </si>
+  <si>
+    <t>Left</t>
+  </si>
+  <si>
+    <t>Izquierda</t>
+  </si>
+  <si>
+    <t>Gauche</t>
+  </si>
+  <si>
+    <t>Links</t>
+  </si>
+  <si>
+    <t>ambi_msg</t>
+  </si>
+  <si>
+    <t>Ambidextrous</t>
+  </si>
+  <si>
+    <t>Ambidiestro/a</t>
+  </si>
+  <si>
+    <t>Ambidextre</t>
+  </si>
+  <si>
+    <t>Beidhändig</t>
+  </si>
+  <si>
+    <t>right_msg</t>
+  </si>
+  <si>
+    <t>Right</t>
+  </si>
+  <si>
+    <t>Derecha</t>
+  </si>
+  <si>
+    <t>Droite</t>
+  </si>
+  <si>
+    <t>Rappel :
+Imaginez À QUOI CELA RESSEMBLE et CE QUE L’ON RESSENT en exécutant vous-même les mouvements décrits dans l’instruction audio.
+Ouvrez les yeux lorsque vous entendez le signal sonore. Décidez aussi RAPIDEMENT ET CORRECTEMENT que possible si l’image affichée correspond à la position finale dans votre imagerie.</t>
+  </si>
+  <si>
+    <t>Rechts</t>
+  </si>
+  <si>
+    <t>There will now be 16 trials in which we will measure your data.
+Each one counts!</t>
+  </si>
+  <si>
+    <t>Es folgen nun 16 Durchgänge, in denen wir Ihre Daten messen möchten.
+Jeder davon zählt!</t>
+  </si>
+  <si>
+    <t>A continuación habrá 16 ensayos en los que mediremos sus datos.
+¡Cada uno cuenta!</t>
+  </si>
+  <si>
+    <t>Il va maintenant y avoir 16 essais au cours desquels nous souhaitons mesurer vos données.
+Chacun d’entre eux compte !</t>
+  </si>
+  <si>
+    <t>You will now hear an audio instruction in 20 trials, each containing 3 to 7 consecutive movements. IMAGINE what it LOOKS LIKE and how it FEELS to perform these movements YOURSELF. Remain seated calmly, CLOSE YOUR EYES and DO NOT MOVE.
 The length of the audio instruction varies randomly. Each audio instruction BEGINS with imagining an upright, standing position. Change your body position IN YOUR IMAGERY according to the instructed movements.
 OPEN your eyes at the SIGNAL TONE. An image of a person seen from behind will appear. Decide as QUICKLY AND ACCURATELY as possible whether the position of this person matches your final position in your imagery.
 Press the ‘S’ key with your left index finger for NO and the ‘L’ key with your right index finger for YES.</t>
   </si>
   <si>
-    <t>Sie hören nun in 36 Durchgängen je eine Audioinstruktion, die 3 bis 7 aufeinanderfolgende Bewegungen enthält. STELLEN SIE SICH VOR, wie es AUSSIEHT und wie es sich ANFÜHLT, diese Bewegungen SELBST auszuführen. Bleiben Sie dabei ruhig sitzen, SCHLIEßEN SIE IHRE AUGEN und BEWEGEN SIE SICH NICHT.
+    <t>Sie hören nun in 20 Durchgängen je eine Audioinstruktion, die 3 bis 7 aufeinanderfolgende Bewegungen enthält. STELLEN SIE SICH VOR, wie es AUSSIEHT und wie es sich ANFÜHLT, diese Bewegungen SELBST auszuführen. Bleiben Sie dabei ruhig sitzen, SCHLIEßEN SIE IHRE AUGEN und BEWEGEN SIE SICH NICHT.
 Die Länge der Audioinstruktion variiert zufällig. Jede Audioinstruktion BEGINNT mit der Vorstellung einer aufrechten, stehenden Position. Verändern Sie IN IHRER VORSTELLUNG Ihre Körperposition entsprechend den instruierten Bewegungen.
 ÖFFNEN Sie Ihre Augen beim SIGNALTON. Es erscheint ein Bild einer Person von hinten. Entscheiden Sie so SCHNELL UND KORREKT wie möglich, ob die Position dieser Person zu Ihrer Endposition in Ihrer Vorstellung passt. 
 Drücken Sie für NEIN die Taste ‚S‘ mit Ihrem linken Zeigefinger und für JA die Taste ‚L‘ mit Ihrem rechten Zeigefinger.</t>
   </si>
   <si>
-    <t>Ahora escuchará en 36 ensayos una instrucción de audio que contiene entre 3 y 7 movimientos consecutivos. IMAGINE cómo SE VE y cómo SE SIENTE realizar estos movimientos USTED MISMO. Permanezca sentado tranquilamente, CIERRE LOS OJOS y NO SE MUEVA.
+    <t>Ahora escuchará en 20 ensayos una instrucción de audio que contiene entre 3 y 7 movimientos consecutivos. IMAGINE cómo SE VE y cómo SE SIENTE realizar estos movimientos USTED MISMO. Permanezca sentado tranquilamente, CIERRE LOS OJOS y NO SE MUEVA.
 La duración de la instrucción de audio varía aleatoriamente. Cada instrucción de audio COMIENZA con la imaginación de una posición erguida, de pie. Modifique la posición de su cuerpo EN SU IMAGINACIÓN de acuerdo con los movimientos instruidos.
 ABRA los ojos al TONO DE SEÑAL. Aparecerá una imagen de una persona vista desde atrás. Decida lo más RÁPIDA Y CORRECTAMENTE posible si la posición de esta persona coincide con su posición final en su imaginación.
 Pulse la tecla ‘S’ con el dedo índice izquierdo para NO y la tecla ‘L’ con el dedo índice derecho para SÍ.</t>
   </si>
   <si>
-    <t>Vous allez maintenant entendre, au cours de 36 essais, une instruction audio contenant 3 à 7 mouvements consécutifs. IMAGINEZ à quoi cela RESSEMBLE et ce que cela FAIT de réaliser VOUS-MÊME ces mouvements. Restez assis calmement, FERMEZ LES YEUX et NE BOUGEZ PAS.
+    <t>Vous allez maintenant entendre, au cours de 20 essais, une instruction audio contenant 3 à 7 mouvements consécutifs. IMAGINEZ à quoi cela RESSEMBLE et ce que cela FAIT de réaliser VOUS-MÊME ces mouvements. Restez assis calmement, FERMEZ LES YEUX et NE BOUGEZ PAS.
 La durée de l’instruction audio varie aléatoirement. Chaque instruction audio COMMENCE par l’imagerie
 d’une position debout et droite. Modifiez votre position corporelle DANS VOTRE IMAGERIE en fonction des mouvements instruits.
 OUVREZ les yeux au SIGNAL SONORE. Une image d’une personne vue de dos apparaît. Décidez aussi VITE ET CORRECTEMENT que possible si la position de cette personne correspond à votre position finale dans votre imagerie.
 Appuyez sur la touche « S » avec l’index gauche pour NON et sur la touche « L » avec l’index droit pour OUI.</t>
   </si>
   <si>
-    <t>You will now hear an audio instruction in 36 trials, each containing 3 to 7 consecutive movements. IMAGINE what it LOOKS LIKE and how it FEELS to perform these movements YOURSELF. Remain seated calmly, CLOSE YOUR EYES and DO NOT MOVE.
+    <t>You will now hear an audio instruction in 20 trials, each containing 3 to 7 consecutive movements. IMAGINE what it LOOKS LIKE and how it FEELS to perform these movements YOURSELF. Remain seated calmly, CLOSE YOUR EYES and DO NOT MOVE.
 The length of the audio instruction varies randomly. Each audio instruction BEGINS with imagining an upright, standing position. Change your body position IN YOUR IMAGERY according to the instructed movements.
 OPEN your eyes at the SIGNAL TONE. An image of a person seen from behind will appear. Decide as QUICKLY AND ACCURATELY as possible whether the position of this person matches your final position in your imagery.
 Press the ‘G’ key with your left middle finger for NO and the ‘H’ key with your left index finger for YES.</t>
   </si>
   <si>
-    <t>When making your decision, pay attention to the rotation of the upper body and to the position of the head, arms, and legs.
-Because the movements build on each other, make sure that when you ROTATE YOUR UPPER BODY, your ARMS and your HEAD ROTATE WITH IT. Your LEGS do NOT rotate.</t>
-  </si>
-  <si>
-    <t>Dies ist das Ende des Experiments.
-Vielen Dank für Ihre Teilnahme!
-Das Experiment schließt sich in 3 Sekunden.</t>
-  </si>
-  <si>
-    <t>Sie hören nun in 36 Durchgängen je eine Audioinstruktion, die 3 bis 7 aufeinanderfolgende Bewegungen enthält. STELLEN SIE SICH VOR, wie es AUSSIEHT und wie es sich ANFÜHLT, diese Bewegungen SELBST auszuführen. Bleiben Sie dabei ruhig sitzen, SCHLIEßEN SIE IHRE AUGEN und BEWEGEN SIE SICH NICHT.
+    <t>Sie hören nun in 20 Durchgängen je eine Audioinstruktion, die 3 bis 7 aufeinanderfolgende Bewegungen enthält. STELLEN SIE SICH VOR, wie es AUSSIEHT und wie es sich ANFÜHLT, diese Bewegungen SELBST auszuführen. Bleiben Sie dabei ruhig sitzen, SCHLIEßEN SIE IHRE AUGEN und BEWEGEN SIE SICH NICHT.
 Die Länge der Audioinstruktion variiert zufällig. Jede Audioinstruktion BEGINNT mit der Vorstellung einer aufrechten, stehenden Position. Verändern Sie IN IHRER VORSTELLUNG Ihre Körperposition entsprechend den instruierten Bewegungen.
 ÖFFNEN Sie Ihre Augen beim SIGNALTON. Es erscheint ein Bild einer Person von hinten. Entscheiden Sie so SCHNELL UND KORREKT wie möglich, ob die Position dieser Person zu Ihrer Endposition in Ihrer Vorstellung passt. 
 Drücken Sie für NEIN die Taste ‚G‘ mit Ihrem linken Mittelfinger und für JA die Taste ‚H‘ mit Ihrem linken Zeigefinger.</t>
   </si>
   <si>
-    <t>Sie hören nun in 36 Durchgängen je eine Audioinstruktion, die 3 bis 7 aufeinanderfolgende Bewegungen enthält. STELLEN SIE SICH VOR, wie es AUSSIEHT und wie es sich ANFÜHLT, diese Bewegungen SELBST auszuführen. Bleiben Sie dabei ruhig sitzen, SCHLIEßEN SIE IHRE AUGEN und BEWEGEN SIE SICH NICHT.
-Die Länge der Audioinstruktion variiert zufällig. Jede Audioinstruktion BEGINNT mit der Vorstellung einer aufrechten, stehenden Position. Verändern Sie IN IHRER VORSTELLUNG Ihre Körperposition entsprechend den instruierten Bewegungen.
-ÖFFNEN Sie Ihre Augen beim SIGNALTON. Es erscheint ein Bild einer Person von hinten. Entscheiden Sie so SCHNELL UND KORREKT wie möglich, ob die Position dieser Person zu Ihrer Endposition in Ihrer Vorstellung passt. 
-Drücken Sie für NEIN die Taste ‚G‘ mit Ihrem rechten Zeigefinger und für JA die Taste ‚H‘ mit Ihrem rechten Mittelfinger.</t>
-  </si>
-  <si>
-    <t>Al tomar su decisión, preste atención a la rotación del tronco, así como a la posición de la cabeza, los brazos y las piernas.
-Dado que los movimientos se encadenan, asegúrese de que, cuando GIRE EL TRONCO, los BRAZOS y la CABEZA GIREN TAMBIÉN. Las PIERNAS, en cambio, NO giran.</t>
-  </si>
-  <si>
-    <t>Ahora escuchará en 36 ensayos una instrucción de audio que contiene entre 3 y 7 movimientos consecutivos. IMAGINE cómo SE VE y cómo SE SIENTE realizar estos movimientos USTED MISMO. Permanezca sentado tranquilamente, CIERRE LOS OJOS y NO SE MUEVA.
-La duración de la instrucción de audio varía aleatoriamente. Cada instrucción de audio COMIENZA con la imaginación de una posición erguida, de pie. Modifique la posición de su cuerpo EN SU IMAGINACIÓN de acuerdo con los movimientos instruidos.
-ABRA los ojos al TONO DE SEÑAL. Aparecerá una imagen de una persona vista desde atrás. Decida lo más RÁPIDA Y CORRECTAMENTE posible si la posición de esta persona coincide con su posición final en su imaginación.
-Pulse la tecla ‘G’ con el dedo índice derecho para NO y la tecla ‘H’ con el dedo medio derecho para SÍ.</t>
-  </si>
-  <si>
-    <t>Ahora escuchará en 36 ensayos una instrucción de audio que contiene entre 3 y 7 movimientos consecutivos. IMAGINE cómo SE VE y cómo SE SIENTE realizar estos movimientos USTED MISMO. Permanezca sentado tranquilamente, CIERRE LOS OJOS y NO SE MUEVA.
+    <t>Ahora escuchará en 20 ensayos una instrucción de audio que contiene entre 3 y 7 movimientos consecutivos. IMAGINE cómo SE VE y cómo SE SIENTE realizar estos movimientos USTED MISMO. Permanezca sentado tranquilamente, CIERRE LOS OJOS y NO SE MUEVA.
 La duración de la instrucción de audio varía aleatoriamente. Cada instrucción de audio COMIENZA con la imaginación de una posición erguida, de pie. Modifique la posición de su cuerpo EN SU IMAGINACIÓN de acuerdo con los movimientos instruidos.
 ABRA los ojos al TONO DE SEÑAL. Aparecerá una imagen de una persona vista desde atrás. Decida lo más RÁPIDA Y CORRECTAMENTE posible si la posición de esta persona coincide con su posición final en su imaginación.
 Pulse la tecla ‘G’ con el dedo medio izquierdo para NO y la tecla ‘H’ con el dedo índice izquierdo para SÍ.</t>
   </si>
   <si>
-    <t>Ceci est la fin de l’expérience.
-Merci pour votre participation.
-L’expérience se terminera dans 3 secondes.</t>
-  </si>
-  <si>
-    <t>Vous allez maintenant entendre, au cours de 36 essais, une instruction audio contenant 3 à 7 mouvements consécutifs. IMAGINEZ à quoi cela RESSEMBLE et ce que cela FAIT de réaliser VOUS-MÊME ces mouvements. Restez assis calmement, FERMEZ LES YEUX et NE BOUGEZ PAS.
+    <t>Vous allez maintenant entendre, au cours de 20 essais, une instruction audio contenant 3 à 7 mouvements consécutifs. IMAGINEZ à quoi cela RESSEMBLE et ce que cela FAIT de réaliser VOUS-MÊME ces mouvements. Restez assis calmement, FERMEZ LES YEUX et NE BOUGEZ PAS.
 La durée de l’instruction audio varie aléatoirement. Chaque instruction audio COMMENCE par l’imagerie
 d’une position debout et droite. Modifiez votre position corporelle DANS VOTRE IMAGERIE en fonction des mouvements instruits.
 OUVREZ les yeux au SIGNAL SONORE. Une image d’une personne vue de dos apparaît. Décidez aussi VITE ET CORRECTEMENT que possible si la position de cette personne correspond à votre position finale dans votre imagerie.
 Appuyez sur la touche « G » avec le majeur gauche pour NON et sur la touche « H » avec l’index gauche pour OUI.</t>
   </si>
   <si>
-    <t>Vous allez maintenant entendre, au cours de 36 essais, une instruction audio contenant 3 à 7 mouvements consécutifs. IMAGINEZ à quoi cela RESSEMBLE et ce que cela FAIT de réaliser VOUS-MÊME ces mouvements. Restez assis calmement, FERMEZ LES YEUX et NE BOUGEZ PAS.
+    <t>You will now hear an audio instruction in 20 trials, each containing 3 to 7 consecutive movements. IMAGINE what it LOOKS LIKE and how it FEELS to perform these movements YOURSELF. Remain seated calmly, CLOSE YOUR EYES and DO NOT MOVE.
+The length of the audio instruction varies randomly. Each audio instruction BEGINS with imagining an upright, standing position. Change your body position IN YOUR IMAGERY according to the instructed movements.
+OPEN your eyes at the SIGNAL TONE. An image of a person seen from behind will appear. Decide as QUICKLY AND ACCURATELY as possible whether the position of this person matches your final position in your imagery.
+Press the ‘G’ key with your right index finger for NO and the ‘H’ key with your right middle finger for YES.</t>
+  </si>
+  <si>
+    <t>Sie hören nun in 20 Durchgängen je eine Audioinstruktion, die 3 bis 7 aufeinanderfolgende Bewegungen enthält. STELLEN SIE SICH VOR, wie es AUSSIEHT und wie es sich ANFÜHLT, diese Bewegungen SELBST auszuführen. Bleiben Sie dabei ruhig sitzen, SCHLIEßEN SIE IHRE AUGEN und BEWEGEN SIE SICH NICHT.
+Die Länge der Audioinstruktion variiert zufällig. Jede Audioinstruktion BEGINNT mit der Vorstellung einer aufrechten, stehenden Position. Verändern Sie IN IHRER VORSTELLUNG Ihre Körperposition entsprechend den instruierten Bewegungen.
+ÖFFNEN Sie Ihre Augen beim SIGNALTON. Es erscheint ein Bild einer Person von hinten. Entscheiden Sie so SCHNELL UND KORREKT wie möglich, ob die Position dieser Person zu Ihrer Endposition in Ihrer Vorstellung passt. 
+Drücken Sie für NEIN die Taste ‚G‘ mit Ihrem rechten Zeigefinger und für JA die Taste ‚H‘ mit Ihrem rechten Mittelfinger.</t>
+  </si>
+  <si>
+    <t>Ahora escuchará en 20 ensayos una instrucción de audio que contiene entre 3 y 7 movimientos consecutivos. IMAGINE cómo SE VE y cómo SE SIENTE realizar estos movimientos USTED MISMO. Permanezca sentado tranquilamente, CIERRE LOS OJOS y NO SE MUEVA.
+La duración de la instrucción de audio varía aleatoriamente. Cada instrucción de audio COMIENZA con la imaginación de una posición erguida, de pie. Modifique la posición de su cuerpo EN SU IMAGINACIÓN de acuerdo con los movimientos instruidos.
+ABRA los ojos al TONO DE SEÑAL. Aparecerá una imagen de una persona vista desde atrás. Decida lo más RÁPIDA Y CORRECTAMENTE posible si la posición de esta persona coincide con su posición final en su imaginación.
+Pulse la tecla ‘G’ con el dedo índice derecho para NO y la tecla ‘H’ con el dedo medio derecho para SÍ.</t>
+  </si>
+  <si>
+    <t>Vous allez maintenant entendre, au cours de 20 essais, une instruction audio contenant 3 à 7 mouvements consécutifs. IMAGINEZ à quoi cela RESSEMBLE et ce que cela FAIT de réaliser VOUS-MÊME ces mouvements. Restez assis calmement, FERMEZ LES YEUX et NE BOUGEZ PAS.
 La durée de l’instruction audio varie aléatoirement. Chaque instruction audio COMMENCE par l’imagerie
 d’une position debout et droite. Modifiez votre position corporelle DANS VOTRE IMAGERIE en fonction des mouvements instruits.
 OUVREZ les yeux au SIGNAL SONORE. Une image d’une personne vue de dos apparaît. Décidez aussi VITE ET CORRECTEMENT que possible si la position de cette personne correspond à votre position finale dans votre imagerie.
 Appuyez sur la touche « G » avec l’index droit pour NON et sur la touche « H » avec le majeur droit pour OUI.</t>
-  </si>
-  <si>
-    <t>Lors de votre décision, prêtez attention à la rotation du haut du corps ainsi qu’à la position de la tête, des bras et des jambes.
-Étant donné que les mouvements s’enchaînent, veillez à ce que, lorsque vous EFFECTUEZ UNE ROTATION DU HAUT DU CORPS, les BRAS et la TÊTE TOURNENT ÉGALEMENT. Les JAMBES, en revanche, ne tournent PAS.</t>
-  </si>
-  <si>
-    <t>You will now hear an audio instruction in 36 trials, each containing 3 to 7 consecutive movements. IMAGINE what it LOOKS LIKE and how it FEELS to perform these movements YOURSELF. Remain seated calmly, CLOSE YOUR EYES and DO NOT MOVE.
-The length of the audio instruction varies randomly. Each audio instruction BEGINS with imagining an upright, standing position. Change your body position IN YOUR IMAGERY according to the instructed movements.
-OPEN your eyes at the SIGNAL TONE. An image of a person seen from behind will appear. Decide as QUICKLY AND ACCURATELY as possible whether the position of this person matches your final position in your imagery.
-Press the ‘G’ key with your right index finger for NO and the ‘H’ key with your right middle finger for YES.</t>
-  </si>
-  <si>
-    <t>Es folgen nun 4 Übungsdurchgänge.</t>
-  </si>
-  <si>
-    <t>Positionieren Sie Ihre Zeigefinger nun auf den Tasten ‚S‘ und ‚L‘ .
-Lassen Sie Ihre Finger auf diesen Tasten ruhen, bis Sie alle Durchgänge der Aufgabe absolviert haben.
-Wenn Sie bereit sind, drücken Sie mit Ihrem Daumen die Leertaste.</t>
-  </si>
-  <si>
-    <t>task_instr_msg_3_bimanual</t>
-  </si>
-  <si>
-    <t>task_instr_msg_3_left</t>
-  </si>
-  <si>
-    <t>task_instr_msg_3_right</t>
-  </si>
-  <si>
-    <t>pract_instr_msg</t>
-  </si>
-  <si>
-    <t>testbl_instr_msg</t>
-  </si>
-  <si>
-    <t>no_feedback_msg</t>
-  </si>
-  <si>
-    <t>Sie werden nun keine Rückmeldungen mehr erhalten.</t>
-  </si>
-  <si>
-    <t>reminder_msg</t>
-  </si>
-  <si>
-    <t>Erinnerung:
-Stellen Sie sich vor, WIE ES AUSSIEHT und WIE ES SICH ANFÜHLT, die in der Audioinstruktion beschriebenen Bewegungen selbst auszuführen.
-Öffnen Sie Ihre Augen beim Signalton. Entscheiden Sie so SCHNELL UND KORREKT wie möglich, ob das gezeigte Bild zu der Endposition in Ihrer Vorstellung passt.</t>
-  </si>
-  <si>
-    <t>Es folgen nun 32 Durchgänge, in denen wir Ihre Daten messen möchten.
-Jeder davon zählt!</t>
-  </si>
-  <si>
-    <t>There will now be 4 practice trials.</t>
-  </si>
-  <si>
-    <t>Now place your index fingers on the ‘S’ and ‘L’ keys.
-Keep your fingers resting on these keys until you have completed all trials of the task.
-When you are ready, press the space bar with your thumb.</t>
-  </si>
-  <si>
-    <t>Positionieren Sie Mittel- und Zeigefinger Ihrer linken Hand nun auf den Tasten ‚G‘ und ‚H‘ .
-Lassen Sie Ihre Finger auf diesen Tasten ruhen, bis Sie alle Durchgänge der Aufgabe absolviert haben.
-Wenn Sie bereit sind, drücken Sie mit Ihrem Daumen die Leertaste.</t>
-  </si>
-  <si>
-    <t>Positionieren Sie Zeige- und Mittelfinger Ihrer rechten Hand nun auf den Tasten ‚G‘ und ‚H‘ .
-Lassen Sie Ihre Finger auf diesen Tasten ruhen, bis Sie alle Durchgänge der Aufgabe absolviert haben.
-Wenn Sie bereit sind, drücken Sie mit Ihrem Daumen die Leertaste.</t>
-  </si>
-  <si>
-    <t>Now place the index and middle fingers of your left hand on the ‘G’ and ‘H’ keys.
-Keep your fingers resting on these keys until you have completed all trials of the task.
-When you are ready, press the space bar with your thumb.</t>
-  </si>
-  <si>
-    <t>Now place the index and middle fingers of your right hand on the ‘G’ and ‘H’ keys.
-Keep your fingers resting on these keys until you have completed all trials of the task.
-When you are ready, press the space bar with your thumb.</t>
-  </si>
-  <si>
-    <t>There will now be 32 trials in which we will measure your data.
-Each one counts!</t>
-  </si>
-  <si>
-    <t>You will now receive no further feedback.</t>
-  </si>
-  <si>
-    <t>Reminder:
-Imagine WHAT IT LOOKS LIKE and HOW IT FEELS to perform the movements described in the audio instruction yourself.
-Open your eyes when you hear the signal tone. Decide as QUICKLY AND ACCURATELY as possible whether the displayed image matches the final position in your imagery.</t>
-  </si>
-  <si>
-    <t>Il va maintenant y avoir 4 essais d’entraînement.</t>
-  </si>
-  <si>
-    <t>Il va maintenant y avoir 32 essais au cours desquels nous souhaitons mesurer vos données.
-Chacun d’entre eux compte !</t>
-  </si>
-  <si>
-    <t>Vous ne recevrez désormais plus aucun retour.</t>
-  </si>
-  <si>
-    <t>A continuación habrá 4 ensayos de práctica.</t>
-  </si>
-  <si>
-    <t>Coloque ahora sus dedos índices sobre las teclas “S” y “L”.
-Mantenga los dedos apoyados sobre estas teclas hasta que haya completado todos los ensayos de la tarea.
-Cuando esté listo/a, presione la barra espaciadora con el pulgar.</t>
-  </si>
-  <si>
-    <t>Coloque ahora el dedo índice y el dedo medio de su mano izquierda sobre las teclas “G” y “H”.
-Mantenga los dedos apoyados sobre estas teclas hasta que haya completado todos los ensayos de la tarea.
-Cuando esté listo/a, presione la barra espaciadora con el pulgar.</t>
-  </si>
-  <si>
-    <t>Coloque ahora el dedo índice y el dedo medio de su mano derecha sobre las teclas “G” y “H”.
-Mantenga los dedos apoyados sobre estas teclas hasta que haya completado todos los ensayos de la tarea.
-Cuando esté listo/a, presione la barra espaciadora con el pulgar.</t>
-  </si>
-  <si>
-    <t>A continuación habrá 32 ensayos en los que mediremos sus datos.
-¡Cada uno cuenta!</t>
-  </si>
-  <si>
-    <t>A partir de ahora no recibirá más retroalimentación.</t>
-  </si>
-  <si>
-    <t>Recordatorio:
-Imagine CÓMO SE VE y CÓMO SE SIENTE ejecutar usted mismo/a los movimientos descritos en la instrucción auditiva.
-Abra los ojos cuando escuche la señal sonora. Decida lo más RÁPIDA Y CORRECTAMENTE posible si la imagen mostrada coincide con la posición final en su imagery.</t>
-  </si>
-  <si>
-    <t>Placez maintenant vos index sur les touches « S » et « L ».
-Laissez vos doigts reposer sur ces touches jusqu’à ce que vous ayez terminé tous les essais de la tâche.
-Lorsque vous êtes prêt(e), appuyez sur la barre d’espace avec votre pouce.</t>
-  </si>
-  <si>
-    <t>Placez maintenant l’index et le majeur de votre main gauche sur les touches « G » et « H ».
-Laissez vos doigts reposer sur ces touches jusqu’à ce que vous ayez terminé tous les essais de la tâche.
-Lorsque vous êtes prêt(e), appuyez sur la barre d’espace avec votre pouce.</t>
-  </si>
-  <si>
-    <t>Placez maintenant l’index et le majeur de votre main droite sur les touches « G » et « H ».
-Laissez vos doigts reposer sur ces touches jusqu’à ce que vous ayez terminé tous les essais de la tâche.
-Lorsque vous êtes prêt(e), appuyez sur la barre d’espace avec votre pouce.</t>
-  </si>
-  <si>
-    <t>you are supposed to imagine how the person in the picture performs the movements.</t>
-  </si>
-  <si>
-    <t>Achten Sie bei Ihrer Entscheidung auf die Drehung des Oberkörpers, die Position des Kopfes, der Arme und Beine.
-Da die Bewegungen aufeinander aufbauen, achten Sie darauf, dass Sie bei DREHUNG IHRES OBERKÖRPERS Ihre ARME und Ihren KOPF MITDREHEN. Ihre BEINE drehen sich dabei NICHT mit.</t>
-  </si>
-  <si>
-    <t>Beispiele:
-&lt;== Neigung des Kopfes nach unten &amp; Drehung des Oberkörpers nach links.
-Anheben des linken Arms in Blickrichtung nach vorne &amp; Drehung des Oberkörpers nach links ==&gt;</t>
-  </si>
-  <si>
-    <t>KORREKTE Antwort</t>
-  </si>
-  <si>
-    <t>CORRECT response</t>
-  </si>
-  <si>
-    <t>INCORRECT response</t>
-  </si>
-  <si>
-    <t>Respuesta CORRECTA</t>
-  </si>
-  <si>
-    <t>Respuesta INCORRECTA</t>
-  </si>
-  <si>
-    <t>Réponse CORRECTE</t>
-  </si>
-  <si>
-    <t>Réponse INCORRECTE</t>
-  </si>
-  <si>
-    <t>fam_msg_1a</t>
-  </si>
-  <si>
-    <t>fam_msg_1b</t>
-  </si>
-  <si>
-    <t>no_movement</t>
-  </si>
-  <si>
-    <t>In the following, you will see 16 images of a person from behind who started in this upright, standing position …</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Im Folgenden sehen Sie 16 Bilder einer Person von hinten, die in dieser aufrechten, stehenden Position startete… </t>
-  </si>
-  <si>
-    <t>A continuación, verá 16 imágenes de una persona vista desde atrás, que comenzó en esta posición erguida y de pie …</t>
-  </si>
-  <si>
-    <t>Dans ce qui suit, vous verrez 16 images d’une personne vue de dos, qui a commencé dans cette position droite et debout …</t>
-  </si>
-  <si>
-    <t>fam_msg_2</t>
-  </si>
-  <si>
-    <t>volume_calib_msg</t>
-  </si>
-  <si>
-    <t>testsound_label</t>
-  </si>
-  <si>
-    <t>In diesem Experiment werden Sie mehrere Audios anhören. Klicken Sie auf ‚Testton abspielen‘ abspielen und stellen Sie die Lautstärke an Ihrem Gerät passend ein.</t>
-  </si>
-  <si>
-    <t>Testton abspielen</t>
-  </si>
-  <si>
-    <t>In this experiment, you will listen to multiple audio recordings. Click on “Play test sound” and adjust the volume on your device accordingly.</t>
-  </si>
-  <si>
-    <t>Play test sound</t>
-  </si>
-  <si>
-    <t>En este experimento, escuchará varios audios. Haga clic en “Reproducir sonido de prueba” y ajuste el volumen de su dispositivo según sea necesario.</t>
-  </si>
-  <si>
-    <t>Reproducir sonido de prueba</t>
-  </si>
-  <si>
-    <t>Dans cette expérience, vous écouterez plusieurs enregistrements audio. Cliquez sur « Lire le son de test » et ajustez le volume de votre appareil en conséquence.</t>
-  </si>
-  <si>
-    <t>Lire le son de test</t>
-  </si>
-  <si>
-    <t>This is the end of the experiment.
-Thank you for participating!
-The experiment finishes in 3 seconds.</t>
-  </si>
-  <si>
-    <t>Este es el final del experimento.
-Gracias por su participación.
-El experimento finalizará en 3 segundos.</t>
-  </si>
-  <si>
-    <t>Unfortunately, your answers were not completely correct.
-Please read the instructions carefully again.</t>
-  </si>
-  <si>
-    <t>testsound</t>
-  </si>
-  <si>
-    <t>Stellen Sie die Lautstärke an Ihrem Gerät so ein, dass Sie dieses Audio klar und deutlich hören können. Bitte lassen Sie die Lautstärke anschließend unverändert. Drücken Sie danach die Leertaste, um fortzufahren.</t>
-  </si>
-  <si>
-    <t>Adjust the volume on your device so that you can hear this audio clearly. Please keep the volume unchanged afterwards. Then press the space bar to continue.</t>
-  </si>
-  <si>
-    <t>Réglez le volume de votre appareil de manière à entendre clairement cet audio. Veuillez ensuite laisser le volume inchangé. Appuyez ensuite sur la barre d’espace pour continuer.</t>
-  </si>
-  <si>
-    <t>Ajuste el volumen de su dispositivo para que pueda escuchar este audio con claridad. Por favor, mantenga el volumen sin cambios a continuación. Luego presione la barra espaciadora para continuar.</t>
-  </si>
-  <si>
-    <t>Raise your right arm forward in the direction of your gaze.</t>
-  </si>
-  <si>
-    <t>Raise your left arm forward in the direction of your gaze.</t>
-  </si>
-  <si>
-    <t>Examples:
-&lt;== Tilting the head downward &amp; rotating the upper body to the left.
-Raising the left arm forward in the direction of gaze &amp; rotating the upper body to the left ==&gt;</t>
-  </si>
-  <si>
-    <t>demographics_msg</t>
-  </si>
-  <si>
-    <t>Please fill out this information about yourself.</t>
-  </si>
-  <si>
-    <t>Por favor completa esta información sobre ti.</t>
-  </si>
-  <si>
-    <t>Veuillez remplir ces informations vous concernant.</t>
-  </si>
-  <si>
-    <t>Bitte füllen Sie diese Informationen über sich selbst aus.</t>
-  </si>
-  <si>
-    <t>age_msg</t>
-  </si>
-  <si>
-    <t>Age:</t>
-  </si>
-  <si>
-    <t>Edad:</t>
-  </si>
-  <si>
-    <t>Âge :</t>
-  </si>
-  <si>
-    <t>Alter:</t>
-  </si>
-  <si>
-    <t>gender_msg</t>
-  </si>
-  <si>
-    <t>Gender:</t>
-  </si>
-  <si>
-    <t>Género</t>
-  </si>
-  <si>
-    <t>Genre :</t>
-  </si>
-  <si>
-    <t>Geschlecht:</t>
-  </si>
-  <si>
-    <t>f_msg</t>
-  </si>
-  <si>
-    <t>Female</t>
-  </si>
-  <si>
-    <t>Mujer</t>
-  </si>
-  <si>
-    <t>Femme</t>
-  </si>
-  <si>
-    <t>Weiblich</t>
-  </si>
-  <si>
-    <t>m_msg</t>
-  </si>
-  <si>
-    <t>Male</t>
-  </si>
-  <si>
-    <t>Hombre</t>
-  </si>
-  <si>
-    <t>Homme</t>
-  </si>
-  <si>
-    <t>Männlich</t>
-  </si>
-  <si>
-    <t>tg_msg</t>
-  </si>
-  <si>
-    <t>Trans-gender</t>
-  </si>
-  <si>
-    <t>Transgénero</t>
-  </si>
-  <si>
-    <t>Transgenre</t>
-  </si>
-  <si>
-    <t>Transgender</t>
-  </si>
-  <si>
-    <t>nb_msg</t>
-  </si>
-  <si>
-    <t>Non-binary</t>
-  </si>
-  <si>
-    <t>No binario</t>
-  </si>
-  <si>
-    <t>Non binaire</t>
-  </si>
-  <si>
-    <t>Nicht-binär</t>
-  </si>
-  <si>
-    <t>o_msg</t>
-  </si>
-  <si>
-    <t>Other</t>
-  </si>
-  <si>
-    <t>Otro</t>
-  </si>
-  <si>
-    <t>Autre</t>
-  </si>
-  <si>
-    <t>Sonstiges</t>
-  </si>
-  <si>
-    <t>pns_msg</t>
-  </si>
-  <si>
-    <t>Prefer not saying</t>
-  </si>
-  <si>
-    <t>Prefiero no decirlo</t>
-  </si>
-  <si>
-    <t>Préfère ne pas le dire</t>
-  </si>
-  <si>
-    <t>Möchte ich nicht sagen</t>
-  </si>
-  <si>
-    <t>next_msg</t>
-  </si>
-  <si>
-    <t>Next</t>
-  </si>
-  <si>
-    <t>Weiter</t>
-  </si>
-  <si>
-    <t>Siguiente</t>
-  </si>
-  <si>
-    <t>Suivant</t>
-  </si>
-  <si>
-    <t>laterality_msg</t>
-  </si>
-  <si>
-    <t>Hand dominance:</t>
-  </si>
-  <si>
-    <t>Mano dominante:</t>
-  </si>
-  <si>
-    <t>Dominance manuelle :</t>
-  </si>
-  <si>
-    <t>Handdominanz:</t>
-  </si>
-  <si>
-    <t>left_msg</t>
-  </si>
-  <si>
-    <t>Left</t>
-  </si>
-  <si>
-    <t>Izquierda</t>
-  </si>
-  <si>
-    <t>Gauche</t>
-  </si>
-  <si>
-    <t>Links</t>
-  </si>
-  <si>
-    <t>ambi_msg</t>
-  </si>
-  <si>
-    <t>Ambidextrous</t>
-  </si>
-  <si>
-    <t>Ambidiestro/a</t>
-  </si>
-  <si>
-    <t>Ambidextre</t>
-  </si>
-  <si>
-    <t>Beidhändig</t>
-  </si>
-  <si>
-    <t>right_msg</t>
-  </si>
-  <si>
-    <t>Right</t>
-  </si>
-  <si>
-    <t>Derecha</t>
-  </si>
-  <si>
-    <t>Droite</t>
-  </si>
-  <si>
-    <t>Rechte</t>
-  </si>
-  <si>
-    <t>Rappel :
-Imaginez À QUOI CELA RESSEMBLE et CE QUE L’ON RESSENT en exécutant vous-même les mouvements décrits dans l’instruction audio.
-Ouvrez les yeux lorsque vous entendez le signal sonore. Décidez aussi RAPIDEMENT ET CORRECTEMENT que possible si l’image affichée correspond à la position finale dans votre imagerie.</t>
   </si>
 </sst>
 </file>
@@ -1305,6 +1305,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1669,89 +1673,89 @@
         <v>4</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>272</v>
+        <v>256</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>273</v>
+        <v>257</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>205</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A5" s="4" t="s">
-        <v>262</v>
+        <v>246</v>
       </c>
       <c r="B5" t="s">
-        <v>266</v>
+        <v>250</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>264</v>
+        <v>248</v>
       </c>
       <c r="D5" t="s">
-        <v>268</v>
+        <v>252</v>
       </c>
       <c r="E5" t="s">
-        <v>270</v>
+        <v>254</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
-        <v>263</v>
+        <v>247</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>267</v>
+        <v>251</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>265</v>
+        <v>249</v>
       </c>
       <c r="D6" t="s">
-        <v>269</v>
+        <v>253</v>
       </c>
       <c r="E6" t="s">
-        <v>271</v>
+        <v>255</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="9" customFormat="1" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A7" s="8" t="s">
-        <v>275</v>
+        <v>259</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>277</v>
+        <v>261</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>276</v>
+        <v>260</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>279</v>
+        <v>263</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>278</v>
+        <v>262</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
-        <v>254</v>
+        <v>238</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>257</v>
+        <v>241</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>258</v>
+        <v>242</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>259</v>
+        <v>243</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>260</v>
+        <v>244</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A9" s="4" t="s">
-        <v>255</v>
+        <v>239</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>10</v>
@@ -1768,7 +1772,7 @@
     </row>
     <row r="10" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
-        <v>261</v>
+        <v>245</v>
       </c>
       <c r="B10" s="4" t="s">
         <v>14</v>
@@ -1802,7 +1806,7 @@
     </row>
     <row r="12" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A12" s="4" t="s">
-        <v>256</v>
+        <v>240</v>
       </c>
       <c r="B12" s="4" t="s">
         <v>23</v>
@@ -1856,7 +1860,7 @@
         <v>37</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>280</v>
+        <v>264</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>38</v>
@@ -1873,7 +1877,7 @@
         <v>41</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>281</v>
+        <v>265</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>42</v>
@@ -2111,16 +2115,16 @@
         <v>142</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>193</v>
+        <v>342</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>194</v>
+        <v>343</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>195</v>
+        <v>344</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>196</v>
+        <v>345</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="156.75" x14ac:dyDescent="0.45">
@@ -2128,16 +2132,16 @@
         <v>143</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>197</v>
+        <v>346</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>200</v>
+        <v>347</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>204</v>
+        <v>348</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>206</v>
+        <v>349</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="156.75" x14ac:dyDescent="0.45">
@@ -2145,16 +2149,16 @@
         <v>144</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>209</v>
+        <v>350</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>201</v>
+        <v>351</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>203</v>
+        <v>352</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>207</v>
+        <v>353</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="71.25" x14ac:dyDescent="0.45">
@@ -2162,16 +2166,16 @@
         <v>145</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>245</v>
+        <v>229</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>208</v>
+        <v>197</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="57" x14ac:dyDescent="0.45">
@@ -2179,10 +2183,10 @@
         <v>146</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>282</v>
+        <v>266</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>246</v>
+        <v>230</v>
       </c>
       <c r="D34" s="4" t="s">
         <v>191</v>
@@ -2264,7 +2268,7 @@
         <v>156</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>244</v>
+        <v>228</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>162</v>
@@ -2349,7 +2353,7 @@
         <v>110</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>274</v>
+        <v>258</v>
       </c>
       <c r="C44" s="4" t="s">
         <v>111</v>
@@ -2366,16 +2370,16 @@
         <v>112</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>248</v>
+        <v>232</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>247</v>
+        <v>231</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>250</v>
+        <v>234</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>252</v>
+        <v>236</v>
       </c>
     </row>
     <row r="46" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
@@ -2383,135 +2387,135 @@
         <v>113</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>249</v>
+        <v>233</v>
       </c>
       <c r="C46" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D46" s="7" t="s">
-        <v>251</v>
+        <v>235</v>
       </c>
       <c r="E46" s="7" t="s">
-        <v>253</v>
+        <v>237</v>
       </c>
     </row>
     <row r="47" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A47" s="4" t="s">
-        <v>215</v>
+        <v>203</v>
       </c>
       <c r="B47" t="s">
-        <v>222</v>
+        <v>209</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>210</v>
+        <v>198</v>
       </c>
       <c r="D47" t="s">
-        <v>234</v>
+        <v>219</v>
       </c>
       <c r="E47" s="7" t="s">
-        <v>231</v>
+        <v>217</v>
       </c>
     </row>
     <row r="48" spans="1:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A48" s="4" t="s">
-        <v>212</v>
+        <v>200</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>223</v>
+        <v>210</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>211</v>
+        <v>199</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>235</v>
+        <v>220</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>241</v>
+        <v>225</v>
       </c>
     </row>
     <row r="49" spans="1:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A49" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B49" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="B49" s="4" t="s">
+      <c r="C49" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="D49" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="E49" s="4" t="s">
         <v>226</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>224</v>
-      </c>
-      <c r="D49" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="E49" s="4" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="50" spans="1:5" ht="42.75" x14ac:dyDescent="0.45">
       <c r="A50" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="B50" s="4" t="s">
         <v>214</v>
       </c>
-      <c r="B50" s="4" t="s">
+      <c r="C50" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="E50" s="4" t="s">
         <v>227</v>
-      </c>
-      <c r="C50" s="4" t="s">
-        <v>225</v>
-      </c>
-      <c r="D50" s="4" t="s">
-        <v>237</v>
-      </c>
-      <c r="E50" s="4" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="51" spans="1:5" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A51" s="4" t="s">
-        <v>216</v>
+        <v>204</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>228</v>
+        <v>338</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>221</v>
+        <v>339</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>238</v>
+        <v>340</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>232</v>
+        <v>341</v>
       </c>
     </row>
     <row r="52" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A52" s="4" t="s">
-        <v>217</v>
+        <v>205</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>229</v>
+        <v>215</v>
       </c>
       <c r="C52" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="D52" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="E52" t="s">
         <v>218</v>
-      </c>
-      <c r="D52" s="7" t="s">
-        <v>239</v>
-      </c>
-      <c r="E52" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="53" spans="1:5" ht="71.25" x14ac:dyDescent="0.45">
       <c r="A53" s="4" t="s">
-        <v>219</v>
+        <v>207</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>230</v>
+        <v>216</v>
       </c>
       <c r="C53" s="4" t="s">
-        <v>220</v>
+        <v>208</v>
       </c>
       <c r="D53" s="4" t="s">
-        <v>240</v>
+        <v>224</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>353</v>
+        <v>336</v>
       </c>
     </row>
     <row r="54" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
@@ -2584,240 +2588,240 @@
     </row>
     <row r="58" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
-        <v>283</v>
+        <v>267</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>284</v>
+        <v>268</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>287</v>
+        <v>271</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>285</v>
+        <v>269</v>
       </c>
       <c r="E58" s="3" t="s">
-        <v>286</v>
+        <v>270</v>
       </c>
     </row>
     <row r="59" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
-        <v>288</v>
+        <v>272</v>
       </c>
       <c r="B59" s="10" t="s">
-        <v>289</v>
+        <v>273</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>292</v>
+        <v>276</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>290</v>
+        <v>274</v>
       </c>
       <c r="E59" s="3" t="s">
-        <v>291</v>
+        <v>275</v>
       </c>
     </row>
     <row r="60" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
-        <v>293</v>
+        <v>277</v>
       </c>
       <c r="B60" s="10" t="s">
-        <v>294</v>
+        <v>278</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>297</v>
+        <v>281</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>295</v>
+        <v>279</v>
       </c>
       <c r="E60" s="3" t="s">
-        <v>296</v>
+        <v>280</v>
       </c>
     </row>
     <row r="61" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
-        <v>298</v>
+        <v>282</v>
       </c>
       <c r="B61" s="10" t="s">
-        <v>299</v>
+        <v>283</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>302</v>
+        <v>286</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>300</v>
+        <v>284</v>
       </c>
       <c r="E61" s="3" t="s">
-        <v>301</v>
+        <v>285</v>
       </c>
     </row>
     <row r="62" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
-        <v>303</v>
+        <v>287</v>
       </c>
       <c r="B62" s="10" t="s">
-        <v>304</v>
+        <v>288</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>307</v>
+        <v>291</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>305</v>
+        <v>289</v>
       </c>
       <c r="E62" s="3" t="s">
-        <v>306</v>
+        <v>290</v>
       </c>
     </row>
     <row r="63" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
-        <v>308</v>
+        <v>292</v>
       </c>
       <c r="B63" s="10" t="s">
-        <v>309</v>
+        <v>293</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>312</v>
+        <v>296</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>310</v>
+        <v>294</v>
       </c>
       <c r="E63" s="3" t="s">
-        <v>311</v>
+        <v>295</v>
       </c>
     </row>
     <row r="64" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
-        <v>313</v>
+        <v>297</v>
       </c>
       <c r="B64" s="10" t="s">
-        <v>314</v>
+        <v>298</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>317</v>
+        <v>301</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>315</v>
+        <v>299</v>
       </c>
       <c r="E64" s="3" t="s">
-        <v>316</v>
+        <v>300</v>
       </c>
     </row>
     <row r="65" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
-        <v>318</v>
+        <v>302</v>
       </c>
       <c r="B65" s="10" t="s">
-        <v>319</v>
+        <v>303</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>322</v>
+        <v>306</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>320</v>
+        <v>304</v>
       </c>
       <c r="E65" s="3" t="s">
-        <v>321</v>
+        <v>305</v>
       </c>
     </row>
     <row r="66" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
-        <v>323</v>
+        <v>307</v>
       </c>
       <c r="B66" s="10" t="s">
-        <v>324</v>
+        <v>308</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>327</v>
+        <v>311</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>325</v>
+        <v>309</v>
       </c>
       <c r="E66" s="3" t="s">
-        <v>326</v>
+        <v>310</v>
       </c>
     </row>
     <row r="67" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
-        <v>333</v>
+        <v>317</v>
       </c>
       <c r="B67" s="10" t="s">
-        <v>334</v>
+        <v>318</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>337</v>
+        <v>321</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>335</v>
+        <v>319</v>
       </c>
       <c r="E67" s="3" t="s">
-        <v>336</v>
+        <v>320</v>
       </c>
     </row>
     <row r="68" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
-        <v>338</v>
+        <v>322</v>
       </c>
       <c r="B68" s="10" t="s">
-        <v>339</v>
+        <v>323</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>342</v>
+        <v>326</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>340</v>
+        <v>324</v>
       </c>
       <c r="E68" s="3" t="s">
-        <v>341</v>
+        <v>325</v>
       </c>
     </row>
     <row r="69" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
-        <v>343</v>
+        <v>327</v>
       </c>
       <c r="B69" s="10" t="s">
-        <v>344</v>
+        <v>328</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>347</v>
+        <v>331</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>345</v>
+        <v>329</v>
       </c>
       <c r="E69" s="3" t="s">
-        <v>346</v>
+        <v>330</v>
       </c>
     </row>
     <row r="70" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
-        <v>348</v>
+        <v>332</v>
       </c>
       <c r="B70" s="10" t="s">
-        <v>349</v>
+        <v>333</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>352</v>
+        <v>337</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>350</v>
+        <v>334</v>
       </c>
       <c r="E70" s="3" t="s">
-        <v>351</v>
+        <v>335</v>
       </c>
     </row>
     <row r="71" spans="1:5" ht="14.25" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
-        <v>328</v>
+        <v>312</v>
       </c>
       <c r="B71" s="10" t="s">
-        <v>329</v>
+        <v>313</v>
       </c>
       <c r="C71" t="s">
-        <v>330</v>
+        <v>314</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>331</v>
+        <v>315</v>
       </c>
       <c r="E71" s="3" t="s">
-        <v>332</v>
+        <v>316</v>
       </c>
     </row>
   </sheetData>
@@ -2838,15 +2842,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B9F5CAB0486A994CA2C3B13E059EF2AE" ma:contentTypeVersion="0" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="8645ec4a60d0c8c7009d2d6675847a91">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="636d7205651659ec4fcda0bcbde9384b">
     <xsd:element name="properties">
@@ -2960,6 +2955,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3725960-8A89-4E70-9C40-340E0EDB6403}">
   <ds:schemaRefs>
@@ -2976,14 +2980,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3744155D-8FAB-4E67-B5E0-C7FDBFB3715D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFF1C174-6AC6-4774-A736-3226A12360E4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2997,4 +2993,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3744155D-8FAB-4E67-B5E0-C7FDBFB3715D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>